<commit_message>
feat(F-NAR-016): TREE-DIF-035 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-035.xlsx
+++ b/stories/arbres/TREE-DIF-035.xlsx
@@ -1197,12 +1197,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Après la pluie, la maison sent le savon. Dans la salle de bain, le carrelage brille. Une goutte tombe encore du robinet. Deux poupées attendent sur le rebord tiède. La poupée de coton a le ventre tout rond. La poupée de bois a les jambes toutes minces. Tu les as sorties du panier ? Oui. Je veux leur donner un bain. Les deux, Chouchou ? Les deux. En ce moment, Chouchou touche le savon. Il sent la lavande, encore un peu froid. Elles ne se ressemblent pas. On les emmène toutes les deux. Le savon, le gobelet, et la serviette. Merci, tu as ouvert le robinet. On prépare, d'abord.</t>
+          <t>Après la pluie, la maison sent le savon. Dans la salle de bain, le carrelage brille. Une goutte tombe encore du robinet. Tu l'entends, Chouchou ? Oui, le robinet. Deux poupées attendent sur le rebord tiède. La poupée de coton a le ventre tout rond. La poupée de bois a les jambes toutes minces. Tu les as sorties du panier ? Oui. Je veux leur donner un bain. Les deux, Chouchou ? Les deux. En ce moment, Chouchou touche le savon. Il sent la lavande, encore un peu froid. Elles ne se ressemblent pas. On les emmène toutes les deux. Le savon, le gobelet, et la serviette. Merci, tu as sorti les deux. On prépare, d'abord.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Après la pluie, la maison sent le savon. Dans la salle de bain, le carrelage brille. Une goutte tombe encore du robinet. Deux poupées attendent sur le rebord tiède. La poupée de coton a le ventre tout rond. La poupée de bois a les jambes toutes minces. Tu les as sorties du panier ? Oui. Je veux leur donner un bain. Les deux, Chouchou ? Les deux. En ce moment, Chouchou touche le savon. Il sent la lavande, encore un peu froid. Elles ne se ressemblent pas. On les emmène toutes les deux. Le savon, le gobelet, et la serviette. Merci, tu as ouvert le robinet. On prépare, d'abord.</t>
+          <t>Après la pluie, la maison sent le savon. Dans la salle de bain, le carrelage brille. Une goutte tombe encore du robinet. Tu l'entends, Chouchou ? Oui, le robinet. Deux poupées attendent sur le rebord tiède. La poupée de coton a le ventre tout rond. La poupée de bois a les jambes toutes minces. Tu les as sorties du panier ? Oui. Je veux leur donner un bain. Les deux, Chouchou ? Les deux. En ce moment, Chouchou touche le savon. Il sent la lavande, encore un peu froid. Elles ne se ressemblent pas. On les emmène toutes les deux. Le savon, le gobelet, et la serviette. Merci, tu as sorti les deux. On prépare, d'abord.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1340,10 +1340,12 @@
           <t>narrateur|Après la pluie, la maison sent le savon.
 narrateur|Dans la salle de bain, le carrelage brille.
 narrateur|Une goutte tombe encore du robinet.
+maman|Tu l'entends, Chouchou ?
+enfant-f|Oui, le robinet.
 narrateur|Deux poupées attendent sur le rebord tiède.
 narrateur|La poupée de coton a le ventre tout rond.
 narrateur|La poupée de bois a les jambes toutes minces.
-maman|Tu les as sorties du panier ?
+papa|Tu les as sorties du panier ?
 enfant-f|Oui.
 enfant-f|Je veux leur donner un bain.
 papa|Les deux, Chouchou ?
@@ -1353,7 +1355,7 @@
 enfant-f|Elles ne se ressemblent pas.
 papa|On les emmène toutes les deux.
 maman|Le savon, le gobelet, et la serviette.
-papa|Merci, tu as ouvert le robinet.
+papa|Merci, tu as sorti les deux.
 enfant-f|On prépare, d'abord.</t>
         </is>
       </c>
@@ -16466,7 +16468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16509,6 +16511,13 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>